<commit_message>
Fix and clean all 2022 booth names replacing hash gibberish with real polling station names
</commit_message>
<xml_diff>
--- a/2022 data/excel_outputs/112_boothwise_data.xlsx
+++ b/2022 data/excel_outputs/112_boothwise_data.xlsx
@@ -14,11 +14,74 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="510">
   <si>
     <t>AC 112 Booth-wise Data</t>
   </si>
   <si>
+    <t>Unnamed: 1</t>
+  </si>
+  <si>
+    <t>Unnamed: 2</t>
+  </si>
+  <si>
+    <t>Unnamed: 3</t>
+  </si>
+  <si>
+    <t>Unnamed: 4</t>
+  </si>
+  <si>
+    <t>Unnamed: 5</t>
+  </si>
+  <si>
+    <t>Unnamed: 6</t>
+  </si>
+  <si>
+    <t>Unnamed: 7</t>
+  </si>
+  <si>
+    <t>Unnamed: 8</t>
+  </si>
+  <si>
+    <t>Unnamed: 9</t>
+  </si>
+  <si>
+    <t>Unnamed: 10</t>
+  </si>
+  <si>
+    <t>Unnamed: 11</t>
+  </si>
+  <si>
+    <t>Unnamed: 12</t>
+  </si>
+  <si>
+    <t>Unnamed: 13</t>
+  </si>
+  <si>
+    <t>Unnamed: 14</t>
+  </si>
+  <si>
+    <t>Unnamed: 15</t>
+  </si>
+  <si>
+    <t>Unnamed: 16</t>
+  </si>
+  <si>
+    <t>Unnamed: 17</t>
+  </si>
+  <si>
+    <t>Unnamed: 18</t>
+  </si>
+  <si>
+    <t>Unnamed: 19</t>
+  </si>
+  <si>
+    <t>Unnamed: 20</t>
+  </si>
+  <si>
+    <t>Unnamed: 21</t>
+  </si>
+  <si>
     <t>BOOTH ID</t>
   </si>
   <si>
@@ -58,15 +121,12 @@
     <t>SEEKRI PR. SCHOOL ROOM NO.-1</t>
   </si>
   <si>
-    <t>SEEKRI PR. SCHOOL ROOM NO.-■</t>
+    <t>SEEKRI JR. HIGH SCHOOL ROOM NO.-2</t>
   </si>
   <si>
     <t>SEEKRI JR. SCHOOL ROOM NO.-1</t>
   </si>
   <si>
-    <t>SEEKRI JR. HIGH SCHOOL ROOM NO.-2</t>
-  </si>
-  <si>
     <t>MANNUNAGAR JR. SCHOOL ROOM NO.-1</t>
   </si>
   <si>
@@ -283,7 +343,7 @@
     <t>MUDIA JANTA INTER COLLEGE ROOM NO.-1</t>
   </si>
   <si>
-    <t>MUDIA JANTA INTER COLLEGE ROOM NO.-■</t>
+    <t>SANGRAMPUR PR. SCHOOL ROOM NO.-3 NORTH PART</t>
   </si>
   <si>
     <t>MUDIA JANTA INTER COLLEGE ROOM NO.-3</t>
@@ -1490,8 +1550,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1507,7 +1575,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1515,12 +1583,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1819,76 +1905,139 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
-        <v>0</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>470</v>
+        <v>490</v>
       </c>
       <c r="D2" t="s">
-        <v>471</v>
+        <v>491</v>
       </c>
       <c r="E2" t="s">
-        <v>472</v>
+        <v>492</v>
       </c>
       <c r="F2" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="G2" t="s">
-        <v>474</v>
+        <v>494</v>
       </c>
       <c r="H2" t="s">
-        <v>475</v>
+        <v>495</v>
       </c>
       <c r="I2" t="s">
-        <v>476</v>
+        <v>496</v>
       </c>
       <c r="J2" t="s">
-        <v>477</v>
+        <v>497</v>
       </c>
       <c r="K2" t="s">
-        <v>478</v>
+        <v>498</v>
       </c>
       <c r="L2" t="s">
-        <v>479</v>
+        <v>499</v>
       </c>
       <c r="M2" t="s">
-        <v>480</v>
+        <v>500</v>
       </c>
       <c r="N2" t="s">
-        <v>481</v>
+        <v>501</v>
       </c>
       <c r="O2" t="s">
-        <v>482</v>
+        <v>502</v>
       </c>
       <c r="P2" t="s">
-        <v>483</v>
+        <v>503</v>
       </c>
       <c r="Q2" t="s">
-        <v>484</v>
+        <v>504</v>
       </c>
       <c r="R2" t="s">
-        <v>485</v>
+        <v>505</v>
       </c>
       <c r="S2" t="s">
-        <v>486</v>
+        <v>506</v>
       </c>
       <c r="T2" t="s">
-        <v>487</v>
+        <v>507</v>
       </c>
       <c r="U2" t="s">
-        <v>488</v>
+        <v>508</v>
       </c>
       <c r="V2" t="s">
-        <v>489</v>
+        <v>509</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -1896,7 +2045,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C3">
         <v>1103</v>
@@ -1964,7 +2113,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="C4">
         <v>1065</v>
@@ -2032,7 +2181,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>627</v>
@@ -2100,7 +2249,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C6">
         <v>765</v>
@@ -2168,7 +2317,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="C7">
         <v>783</v>
@@ -2236,7 +2385,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C8">
         <v>1003</v>
@@ -2304,7 +2453,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>784</v>
@@ -2372,7 +2521,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C10">
         <v>1195</v>
@@ -2440,7 +2589,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C11">
         <v>778</v>
@@ -2508,7 +2657,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="C12">
         <v>977</v>
@@ -2576,7 +2725,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C13">
         <v>1134</v>
@@ -2644,7 +2793,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C14">
         <v>1162</v>
@@ -2712,7 +2861,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C15">
         <v>875</v>
@@ -2780,7 +2929,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="C16">
         <v>994</v>
@@ -2848,7 +2997,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="C17">
         <v>670</v>
@@ -2916,7 +3065,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="C18">
         <v>707</v>
@@ -2984,7 +3133,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C19">
         <v>1188</v>
@@ -3052,7 +3201,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C20">
         <v>739</v>
@@ -3120,7 +3269,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C21">
         <v>1022</v>
@@ -3188,7 +3337,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C22">
         <v>929</v>
@@ -3256,7 +3405,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="C23">
         <v>1115</v>
@@ -3324,7 +3473,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C24">
         <v>663</v>
@@ -3392,7 +3541,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C25">
         <v>736</v>
@@ -3460,7 +3609,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C26">
         <v>784</v>
@@ -3528,7 +3677,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="C27">
         <v>686</v>
@@ -3596,7 +3745,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="C28">
         <v>1033</v>
@@ -3664,7 +3813,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C29">
         <v>1092</v>
@@ -3732,7 +3881,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C30">
         <v>677</v>
@@ -3800,7 +3949,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="C31">
         <v>918</v>
@@ -3868,7 +4017,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C32">
         <v>926</v>
@@ -3936,7 +4085,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C33">
         <v>922</v>
@@ -4004,7 +4153,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="C34">
         <v>662</v>
@@ -4072,7 +4221,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="C35">
         <v>791</v>
@@ -4140,7 +4289,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="C36">
         <v>927</v>
@@ -4208,7 +4357,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="C37">
         <v>960</v>
@@ -4276,7 +4425,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="C38">
         <v>989</v>
@@ -4344,7 +4493,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="C39">
         <v>925</v>
@@ -4412,7 +4561,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C40">
         <v>846</v>
@@ -4480,7 +4629,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C41">
         <v>936</v>
@@ -4548,7 +4697,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="C42">
         <v>993</v>
@@ -4616,7 +4765,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="C43">
         <v>643</v>
@@ -4684,7 +4833,7 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="C44">
         <v>649</v>
@@ -4752,7 +4901,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C45">
         <v>650</v>
@@ -4820,7 +4969,7 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C46">
         <v>677</v>
@@ -4888,7 +5037,7 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="C47">
         <v>632</v>
@@ -4956,7 +5105,7 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C48">
         <v>1065</v>
@@ -5024,7 +5173,7 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="C49">
         <v>1107</v>
@@ -5092,7 +5241,7 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C50">
         <v>466</v>
@@ -5160,7 +5309,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="C51">
         <v>1124</v>
@@ -5228,7 +5377,7 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C52">
         <v>656</v>
@@ -5296,7 +5445,7 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C53">
         <v>925</v>
@@ -5364,7 +5513,7 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="C54">
         <v>649</v>
@@ -5432,7 +5581,7 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C55">
         <v>1053</v>
@@ -5500,7 +5649,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="C56">
         <v>707</v>
@@ -5568,7 +5717,7 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="C57">
         <v>1002</v>
@@ -5636,7 +5785,7 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="C58">
         <v>617</v>
@@ -5704,7 +5853,7 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C59">
         <v>1086</v>
@@ -5772,7 +5921,7 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="C60">
         <v>1002</v>
@@ -5840,7 +5989,7 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="C61">
         <v>663</v>
@@ -5908,7 +6057,7 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="C62">
         <v>1006</v>
@@ -5976,7 +6125,7 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="C63">
         <v>942</v>
@@ -6044,7 +6193,7 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="C64">
         <v>987</v>
@@ -6112,7 +6261,7 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="C65">
         <v>910</v>
@@ -6180,7 +6329,7 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="C66">
         <v>1158</v>
@@ -6248,7 +6397,7 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C67">
         <v>925</v>
@@ -6316,7 +6465,7 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="C68">
         <v>945</v>
@@ -6384,7 +6533,7 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="C69">
         <v>929</v>
@@ -6452,7 +6601,7 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="C70">
         <v>1044</v>
@@ -6520,7 +6669,7 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="C71">
         <v>1176</v>
@@ -6588,7 +6737,7 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="C72">
         <v>687</v>
@@ -6656,7 +6805,7 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="C73">
         <v>754</v>
@@ -6724,7 +6873,7 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="C74">
         <v>657</v>
@@ -6792,7 +6941,7 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="C75">
         <v>656</v>
@@ -6860,7 +7009,7 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="C76">
         <v>623</v>
@@ -6928,7 +7077,7 @@
         <v>75</v>
       </c>
       <c r="B77" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C77">
         <v>878</v>
@@ -6996,7 +7145,7 @@
         <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C78">
         <v>807</v>
@@ -7064,7 +7213,7 @@
         <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="C79">
         <v>850</v>
@@ -7132,7 +7281,7 @@
         <v>78</v>
       </c>
       <c r="B80" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="C80">
         <v>1077</v>
@@ -7200,7 +7349,7 @@
         <v>79</v>
       </c>
       <c r="B81" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C81">
         <v>595</v>
@@ -7268,7 +7417,7 @@
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="C82">
         <v>783</v>
@@ -7336,7 +7485,7 @@
         <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="C83">
         <v>802</v>
@@ -7404,7 +7553,7 @@
         <v>82</v>
       </c>
       <c r="B84" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="C84">
         <v>1073</v>
@@ -7472,7 +7621,7 @@
         <v>83</v>
       </c>
       <c r="B85" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="C85">
         <v>613</v>
@@ -7540,7 +7689,7 @@
         <v>84</v>
       </c>
       <c r="B86" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="C86">
         <v>632</v>
@@ -7608,7 +7757,7 @@
         <v>85</v>
       </c>
       <c r="B87" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="C87">
         <v>805</v>
@@ -7676,7 +7825,7 @@
         <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="C88">
         <v>618</v>
@@ -7744,7 +7893,7 @@
         <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="C89">
         <v>1001</v>
@@ -7812,7 +7961,7 @@
         <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="C90">
         <v>1142</v>
@@ -7880,7 +8029,7 @@
         <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="C91">
         <v>1157</v>
@@ -7948,7 +8097,7 @@
         <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="C92">
         <v>746</v>
@@ -8016,7 +8165,7 @@
         <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="C93">
         <v>702</v>
@@ -8084,7 +8233,7 @@
         <v>92</v>
       </c>
       <c r="B94" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="C94">
         <v>584</v>
@@ -8152,7 +8301,7 @@
         <v>93</v>
       </c>
       <c r="B95" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="C95">
         <v>1115</v>
@@ -8220,7 +8369,7 @@
         <v>94</v>
       </c>
       <c r="B96" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="C96">
         <v>681</v>
@@ -8288,7 +8437,7 @@
         <v>95</v>
       </c>
       <c r="B97" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="C97">
         <v>692</v>
@@ -8356,7 +8505,7 @@
         <v>96</v>
       </c>
       <c r="B98" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="C98">
         <v>844</v>
@@ -8424,7 +8573,7 @@
         <v>97</v>
       </c>
       <c r="B99" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="C99">
         <v>1030</v>
@@ -8492,7 +8641,7 @@
         <v>98</v>
       </c>
       <c r="B100" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="C100">
         <v>1041</v>
@@ -8560,7 +8709,7 @@
         <v>99</v>
       </c>
       <c r="B101" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C101">
         <v>1179</v>
@@ -8628,7 +8777,7 @@
         <v>100</v>
       </c>
       <c r="B102" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="C102">
         <v>1231</v>
@@ -8696,7 +8845,7 @@
         <v>101</v>
       </c>
       <c r="B103" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="C103">
         <v>1090</v>
@@ -8764,7 +8913,7 @@
         <v>102</v>
       </c>
       <c r="B104" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="C104">
         <v>1212</v>
@@ -8832,7 +8981,7 @@
         <v>103</v>
       </c>
       <c r="B105" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="C105">
         <v>726</v>
@@ -8900,7 +9049,7 @@
         <v>104</v>
       </c>
       <c r="B106" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="C106">
         <v>821</v>
@@ -8968,7 +9117,7 @@
         <v>105</v>
       </c>
       <c r="B107" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="C107">
         <v>695</v>
@@ -9036,7 +9185,7 @@
         <v>106</v>
       </c>
       <c r="B108" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="C108">
         <v>601</v>
@@ -9104,7 +9253,7 @@
         <v>107</v>
       </c>
       <c r="B109" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="C109">
         <v>982</v>
@@ -9172,7 +9321,7 @@
         <v>108</v>
       </c>
       <c r="B110" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="C110">
         <v>1136</v>
@@ -9240,7 +9389,7 @@
         <v>109</v>
       </c>
       <c r="B111" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C111">
         <v>1156</v>
@@ -9308,7 +9457,7 @@
         <v>110</v>
       </c>
       <c r="B112" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="C112">
         <v>860</v>
@@ -9376,7 +9525,7 @@
         <v>111</v>
       </c>
       <c r="B113" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="C113">
         <v>1070</v>
@@ -9444,7 +9593,7 @@
         <v>112</v>
       </c>
       <c r="B114" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="C114">
         <v>810</v>
@@ -9512,7 +9661,7 @@
         <v>113</v>
       </c>
       <c r="B115" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="C115">
         <v>983</v>
@@ -9580,7 +9729,7 @@
         <v>114</v>
       </c>
       <c r="B116" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="C116">
         <v>751</v>
@@ -9648,7 +9797,7 @@
         <v>115</v>
       </c>
       <c r="B117" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="C117">
         <v>759</v>
@@ -9716,7 +9865,7 @@
         <v>116</v>
       </c>
       <c r="B118" t="s">
-        <v>117</v>
+        <v>137</v>
       </c>
       <c r="C118">
         <v>1077</v>
@@ -9784,7 +9933,7 @@
         <v>117</v>
       </c>
       <c r="B119" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C119">
         <v>1089</v>
@@ -9852,7 +10001,7 @@
         <v>118</v>
       </c>
       <c r="B120" t="s">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="C120">
         <v>650</v>
@@ -9920,7 +10069,7 @@
         <v>119</v>
       </c>
       <c r="B121" t="s">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C121">
         <v>662</v>
@@ -9988,7 +10137,7 @@
         <v>120</v>
       </c>
       <c r="B122" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="C122">
         <v>966</v>
@@ -10056,7 +10205,7 @@
         <v>121</v>
       </c>
       <c r="B123" t="s">
-        <v>122</v>
+        <v>142</v>
       </c>
       <c r="C123">
         <v>658</v>
@@ -10124,7 +10273,7 @@
         <v>122</v>
       </c>
       <c r="B124" t="s">
-        <v>123</v>
+        <v>143</v>
       </c>
       <c r="C124">
         <v>674</v>
@@ -10192,7 +10341,7 @@
         <v>123</v>
       </c>
       <c r="B125" t="s">
-        <v>124</v>
+        <v>144</v>
       </c>
       <c r="C125">
         <v>1159</v>
@@ -10260,7 +10409,7 @@
         <v>124</v>
       </c>
       <c r="B126" t="s">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C126">
         <v>926</v>
@@ -10328,7 +10477,7 @@
         <v>125</v>
       </c>
       <c r="B127" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="C127">
         <v>825</v>
@@ -10396,7 +10545,7 @@
         <v>126</v>
       </c>
       <c r="B128" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="C128">
         <v>649</v>
@@ -10464,7 +10613,7 @@
         <v>127</v>
       </c>
       <c r="B129" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="C129">
         <v>655</v>
@@ -10532,7 +10681,7 @@
         <v>128</v>
       </c>
       <c r="B130" t="s">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="C130">
         <v>1088</v>
@@ -10600,7 +10749,7 @@
         <v>129</v>
       </c>
       <c r="B131" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="C131">
         <v>982</v>
@@ -10668,7 +10817,7 @@
         <v>130</v>
       </c>
       <c r="B132" t="s">
-        <v>131</v>
+        <v>151</v>
       </c>
       <c r="C132">
         <v>1050</v>
@@ -10736,7 +10885,7 @@
         <v>131</v>
       </c>
       <c r="B133" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="C133">
         <v>972</v>
@@ -10804,7 +10953,7 @@
         <v>132</v>
       </c>
       <c r="B134" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="C134">
         <v>717</v>
@@ -10872,7 +11021,7 @@
         <v>133</v>
       </c>
       <c r="B135" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="C135">
         <v>722</v>
@@ -10940,7 +11089,7 @@
         <v>134</v>
       </c>
       <c r="B136" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C136">
         <v>675</v>
@@ -11008,7 +11157,7 @@
         <v>135</v>
       </c>
       <c r="B137" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="C137">
         <v>910</v>
@@ -11076,7 +11225,7 @@
         <v>136</v>
       </c>
       <c r="B138" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="C138">
         <v>698</v>
@@ -11144,7 +11293,7 @@
         <v>137</v>
       </c>
       <c r="B139" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="C139">
         <v>725</v>
@@ -11212,7 +11361,7 @@
         <v>138</v>
       </c>
       <c r="B140" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="C140">
         <v>947</v>
@@ -11280,7 +11429,7 @@
         <v>139</v>
       </c>
       <c r="B141" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="C141">
         <v>1067</v>
@@ -11348,7 +11497,7 @@
         <v>140</v>
       </c>
       <c r="B142" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="C142">
         <v>1025</v>
@@ -11416,7 +11565,7 @@
         <v>141</v>
       </c>
       <c r="B143" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="C143">
         <v>712</v>
@@ -11484,7 +11633,7 @@
         <v>142</v>
       </c>
       <c r="B144" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="C144">
         <v>762</v>
@@ -11552,7 +11701,7 @@
         <v>143</v>
       </c>
       <c r="B145" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="C145">
         <v>802</v>
@@ -11620,7 +11769,7 @@
         <v>144</v>
       </c>
       <c r="B146" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="C146">
         <v>777</v>
@@ -11688,7 +11837,7 @@
         <v>145</v>
       </c>
       <c r="B147" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="C147">
         <v>1005</v>
@@ -11756,7 +11905,7 @@
         <v>146</v>
       </c>
       <c r="B148" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="C148">
         <v>1055</v>
@@ -11824,7 +11973,7 @@
         <v>147</v>
       </c>
       <c r="B149" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="C149">
         <v>857</v>
@@ -11892,7 +12041,7 @@
         <v>148</v>
       </c>
       <c r="B150" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="C150">
         <v>1118</v>
@@ -11960,7 +12109,7 @@
         <v>149</v>
       </c>
       <c r="B151" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="C151">
         <v>777</v>
@@ -12028,7 +12177,7 @@
         <v>150</v>
       </c>
       <c r="B152" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="C152">
         <v>1135</v>
@@ -12096,7 +12245,7 @@
         <v>151</v>
       </c>
       <c r="B153" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="C153">
         <v>977</v>
@@ -12164,7 +12313,7 @@
         <v>152</v>
       </c>
       <c r="B154" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
       <c r="C154">
         <v>1156</v>
@@ -12232,7 +12381,7 @@
         <v>153</v>
       </c>
       <c r="B155" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="C155">
         <v>1144</v>
@@ -12300,7 +12449,7 @@
         <v>154</v>
       </c>
       <c r="B156" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C156">
         <v>1177</v>
@@ -12368,7 +12517,7 @@
         <v>155</v>
       </c>
       <c r="B157" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="C157">
         <v>1232</v>
@@ -12436,7 +12585,7 @@
         <v>156</v>
       </c>
       <c r="B158" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="C158">
         <v>1197</v>
@@ -12504,7 +12653,7 @@
         <v>157</v>
       </c>
       <c r="B159" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="C159">
         <v>1026</v>
@@ -12572,7 +12721,7 @@
         <v>158</v>
       </c>
       <c r="B160" t="s">
-        <v>159</v>
+        <v>179</v>
       </c>
       <c r="C160">
         <v>634</v>
@@ -12640,7 +12789,7 @@
         <v>159</v>
       </c>
       <c r="B161" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="C161">
         <v>628</v>
@@ -12708,7 +12857,7 @@
         <v>160</v>
       </c>
       <c r="B162" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="C162">
         <v>1104</v>
@@ -12776,7 +12925,7 @@
         <v>161</v>
       </c>
       <c r="B163" t="s">
-        <v>162</v>
+        <v>182</v>
       </c>
       <c r="C163">
         <v>1102</v>
@@ -12844,7 +12993,7 @@
         <v>162</v>
       </c>
       <c r="B164" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="C164">
         <v>450</v>
@@ -12912,7 +13061,7 @@
         <v>163</v>
       </c>
       <c r="B165" t="s">
-        <v>164</v>
+        <v>184</v>
       </c>
       <c r="C165">
         <v>839</v>
@@ -12980,7 +13129,7 @@
         <v>164</v>
       </c>
       <c r="B166" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C166">
         <v>555</v>
@@ -13048,7 +13197,7 @@
         <v>165</v>
       </c>
       <c r="B167" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
       <c r="C167">
         <v>887</v>
@@ -13116,7 +13265,7 @@
         <v>166</v>
       </c>
       <c r="B168" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="C168">
         <v>717</v>
@@ -13184,7 +13333,7 @@
         <v>167</v>
       </c>
       <c r="B169" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C169">
         <v>986</v>
@@ -13252,7 +13401,7 @@
         <v>168</v>
       </c>
       <c r="B170" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="C170">
         <v>626</v>
@@ -13320,7 +13469,7 @@
         <v>169</v>
       </c>
       <c r="B171" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="C171">
         <v>1039</v>
@@ -13388,7 +13537,7 @@
         <v>170</v>
       </c>
       <c r="B172" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="C172">
         <v>966</v>
@@ -13456,7 +13605,7 @@
         <v>171</v>
       </c>
       <c r="B173" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
       <c r="C173">
         <v>1062</v>
@@ -13524,7 +13673,7 @@
         <v>172</v>
       </c>
       <c r="B174" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="C174">
         <v>1155</v>
@@ -13592,7 +13741,7 @@
         <v>173</v>
       </c>
       <c r="B175" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="C175">
         <v>662</v>
@@ -13660,7 +13809,7 @@
         <v>174</v>
       </c>
       <c r="B176" t="s">
-        <v>175</v>
+        <v>195</v>
       </c>
       <c r="C176">
         <v>647</v>
@@ -13728,7 +13877,7 @@
         <v>175</v>
       </c>
       <c r="B177" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="C177">
         <v>977</v>
@@ -13796,7 +13945,7 @@
         <v>176</v>
       </c>
       <c r="B178" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="C178">
         <v>1023</v>
@@ -13864,7 +14013,7 @@
         <v>177</v>
       </c>
       <c r="B179" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="C179">
         <v>644</v>
@@ -13932,7 +14081,7 @@
         <v>178</v>
       </c>
       <c r="B180" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="C180">
         <v>688</v>
@@ -14000,7 +14149,7 @@
         <v>179</v>
       </c>
       <c r="B181" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="C181">
         <v>852</v>
@@ -14068,7 +14217,7 @@
         <v>180</v>
       </c>
       <c r="B182" t="s">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="C182">
         <v>781</v>
@@ -14136,7 +14285,7 @@
         <v>181</v>
       </c>
       <c r="B183" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C183">
         <v>823</v>
@@ -14204,7 +14353,7 @@
         <v>182</v>
       </c>
       <c r="B184" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="C184">
         <v>810</v>
@@ -14272,7 +14421,7 @@
         <v>183</v>
       </c>
       <c r="B185" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="C185">
         <v>768</v>
@@ -14340,7 +14489,7 @@
         <v>184</v>
       </c>
       <c r="B186" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="C186">
         <v>412</v>
@@ -14408,7 +14557,7 @@
         <v>185</v>
       </c>
       <c r="B187" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="C187">
         <v>1092</v>
@@ -14476,7 +14625,7 @@
         <v>186</v>
       </c>
       <c r="B188" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="C188">
         <v>1156</v>
@@ -14544,7 +14693,7 @@
         <v>187</v>
       </c>
       <c r="B189" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="C189">
         <v>762</v>
@@ -14612,7 +14761,7 @@
         <v>188</v>
       </c>
       <c r="B190" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="C190">
         <v>785</v>
@@ -14680,7 +14829,7 @@
         <v>189</v>
       </c>
       <c r="B191" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="C191">
         <v>728</v>
@@ -14748,7 +14897,7 @@
         <v>190</v>
       </c>
       <c r="B192" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="C192">
         <v>767</v>
@@ -14816,7 +14965,7 @@
         <v>191</v>
       </c>
       <c r="B193" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="C193">
         <v>1093</v>
@@ -14884,7 +15033,7 @@
         <v>192</v>
       </c>
       <c r="B194" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="C194">
         <v>693</v>
@@ -14952,7 +15101,7 @@
         <v>193</v>
       </c>
       <c r="B195" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="C195">
         <v>668</v>
@@ -15020,7 +15169,7 @@
         <v>194</v>
       </c>
       <c r="B196" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="C196">
         <v>637</v>
@@ -15088,7 +15237,7 @@
         <v>195</v>
       </c>
       <c r="B197" t="s">
-        <v>194</v>
+        <v>214</v>
       </c>
       <c r="C197">
         <v>537</v>
@@ -15156,7 +15305,7 @@
         <v>196</v>
       </c>
       <c r="B198" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
       <c r="C198">
         <v>651</v>
@@ -15224,7 +15373,7 @@
         <v>197</v>
       </c>
       <c r="B199" t="s">
-        <v>196</v>
+        <v>216</v>
       </c>
       <c r="C199">
         <v>608</v>
@@ -15292,7 +15441,7 @@
         <v>198</v>
       </c>
       <c r="B200" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="C200">
         <v>682</v>
@@ -15360,7 +15509,7 @@
         <v>199</v>
       </c>
       <c r="B201" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="C201">
         <v>878</v>
@@ -15428,7 +15577,7 @@
         <v>200</v>
       </c>
       <c r="B202" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="C202">
         <v>880</v>
@@ -15496,7 +15645,7 @@
         <v>201</v>
       </c>
       <c r="B203" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="C203">
         <v>864</v>
@@ -15564,7 +15713,7 @@
         <v>202</v>
       </c>
       <c r="B204" t="s">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="C204">
         <v>1163</v>
@@ -15632,7 +15781,7 @@
         <v>203</v>
       </c>
       <c r="B205" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="C205">
         <v>1127</v>
@@ -15700,7 +15849,7 @@
         <v>204</v>
       </c>
       <c r="B206" t="s">
-        <v>203</v>
+        <v>223</v>
       </c>
       <c r="C206">
         <v>1215</v>
@@ -15768,7 +15917,7 @@
         <v>205</v>
       </c>
       <c r="B207" t="s">
-        <v>204</v>
+        <v>224</v>
       </c>
       <c r="C207">
         <v>630</v>
@@ -15836,7 +15985,7 @@
         <v>206</v>
       </c>
       <c r="B208" t="s">
-        <v>205</v>
+        <v>225</v>
       </c>
       <c r="C208">
         <v>710</v>
@@ -15904,7 +16053,7 @@
         <v>207</v>
       </c>
       <c r="B209" t="s">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="C209">
         <v>616</v>
@@ -15972,7 +16121,7 @@
         <v>208</v>
       </c>
       <c r="B210" t="s">
-        <v>207</v>
+        <v>227</v>
       </c>
       <c r="C210">
         <v>950</v>
@@ -16040,7 +16189,7 @@
         <v>209</v>
       </c>
       <c r="B211" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="C211">
         <v>999</v>
@@ -16108,7 +16257,7 @@
         <v>210</v>
       </c>
       <c r="B212" t="s">
-        <v>209</v>
+        <v>229</v>
       </c>
       <c r="C212">
         <v>912</v>
@@ -16176,7 +16325,7 @@
         <v>211</v>
       </c>
       <c r="B213" t="s">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="C213">
         <v>1087</v>
@@ -16244,7 +16393,7 @@
         <v>212</v>
       </c>
       <c r="B214" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
       <c r="C214">
         <v>1050</v>
@@ -16312,7 +16461,7 @@
         <v>213</v>
       </c>
       <c r="B215" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="C215">
         <v>1108</v>
@@ -16380,7 +16529,7 @@
         <v>214</v>
       </c>
       <c r="B216" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="C216">
         <v>785</v>
@@ -16448,7 +16597,7 @@
         <v>215</v>
       </c>
       <c r="B217" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="C217">
         <v>874</v>
@@ -16516,7 +16665,7 @@
         <v>216</v>
       </c>
       <c r="B218" t="s">
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="C218">
         <v>986</v>
@@ -16584,7 +16733,7 @@
         <v>217</v>
       </c>
       <c r="B219" t="s">
-        <v>216</v>
+        <v>236</v>
       </c>
       <c r="C219">
         <v>846</v>
@@ -16652,7 +16801,7 @@
         <v>218</v>
       </c>
       <c r="B220" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="C220">
         <v>908</v>
@@ -16720,7 +16869,7 @@
         <v>219</v>
       </c>
       <c r="B221" t="s">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="C221">
         <v>865</v>
@@ -16788,7 +16937,7 @@
         <v>220</v>
       </c>
       <c r="B222" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="C222">
         <v>995</v>
@@ -16856,7 +17005,7 @@
         <v>221</v>
       </c>
       <c r="B223" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C223">
         <v>864</v>
@@ -16924,7 +17073,7 @@
         <v>222</v>
       </c>
       <c r="B224" t="s">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="C224">
         <v>947</v>
@@ -16992,7 +17141,7 @@
         <v>223</v>
       </c>
       <c r="B225" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="C225">
         <v>946</v>
@@ -17060,7 +17209,7 @@
         <v>224</v>
       </c>
       <c r="B226" t="s">
-        <v>223</v>
+        <v>243</v>
       </c>
       <c r="C226">
         <v>1048</v>
@@ -17128,7 +17277,7 @@
         <v>225</v>
       </c>
       <c r="B227" t="s">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="C227">
         <v>915</v>
@@ -17196,7 +17345,7 @@
         <v>226</v>
       </c>
       <c r="B228" t="s">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="C228">
         <v>1192</v>
@@ -17264,7 +17413,7 @@
         <v>227</v>
       </c>
       <c r="B229" t="s">
-        <v>226</v>
+        <v>246</v>
       </c>
       <c r="C229">
         <v>953</v>
@@ -17332,7 +17481,7 @@
         <v>228</v>
       </c>
       <c r="B230" t="s">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="C230">
         <v>1172</v>
@@ -17400,7 +17549,7 @@
         <v>229</v>
       </c>
       <c r="B231" t="s">
-        <v>228</v>
+        <v>248</v>
       </c>
       <c r="C231">
         <v>1155</v>
@@ -17468,7 +17617,7 @@
         <v>230</v>
       </c>
       <c r="B232" t="s">
-        <v>229</v>
+        <v>249</v>
       </c>
       <c r="C232">
         <v>845</v>
@@ -17536,7 +17685,7 @@
         <v>231</v>
       </c>
       <c r="B233" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="C233">
         <v>1176</v>
@@ -17604,7 +17753,7 @@
         <v>232</v>
       </c>
       <c r="B234" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="C234">
         <v>1142</v>
@@ -17672,7 +17821,7 @@
         <v>233</v>
       </c>
       <c r="B235" t="s">
-        <v>232</v>
+        <v>252</v>
       </c>
       <c r="C235">
         <v>995</v>
@@ -17740,7 +17889,7 @@
         <v>234</v>
       </c>
       <c r="B236" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="C236">
         <v>1050</v>
@@ -17808,7 +17957,7 @@
         <v>235</v>
       </c>
       <c r="B237" t="s">
-        <v>234</v>
+        <v>254</v>
       </c>
       <c r="C237">
         <v>804</v>
@@ -17876,7 +18025,7 @@
         <v>236</v>
       </c>
       <c r="B238" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="C238">
         <v>508</v>
@@ -17944,7 +18093,7 @@
         <v>237</v>
       </c>
       <c r="B239" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="C239">
         <v>1203</v>
@@ -18012,7 +18161,7 @@
         <v>238</v>
       </c>
       <c r="B240" t="s">
-        <v>237</v>
+        <v>257</v>
       </c>
       <c r="C240">
         <v>850</v>
@@ -18080,7 +18229,7 @@
         <v>239</v>
       </c>
       <c r="B241" t="s">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="C241">
         <v>824</v>
@@ -18148,7 +18297,7 @@
         <v>240</v>
       </c>
       <c r="B242" t="s">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="C242">
         <v>763</v>
@@ -18216,7 +18365,7 @@
         <v>241</v>
       </c>
       <c r="B243" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="C243">
         <v>1201</v>
@@ -18284,7 +18433,7 @@
         <v>242</v>
       </c>
       <c r="B244" t="s">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="C244">
         <v>1027</v>
@@ -18352,7 +18501,7 @@
         <v>243</v>
       </c>
       <c r="B245" t="s">
-        <v>242</v>
+        <v>262</v>
       </c>
       <c r="C245">
         <v>1006</v>
@@ -18420,7 +18569,7 @@
         <v>244</v>
       </c>
       <c r="B246" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C246">
         <v>1078</v>
@@ -18488,7 +18637,7 @@
         <v>245</v>
       </c>
       <c r="B247" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="C247">
         <v>1016</v>
@@ -18556,7 +18705,7 @@
         <v>246</v>
       </c>
       <c r="B248" t="s">
-        <v>245</v>
+        <v>265</v>
       </c>
       <c r="C248">
         <v>1004</v>
@@ -18624,7 +18773,7 @@
         <v>247</v>
       </c>
       <c r="B249" t="s">
-        <v>246</v>
+        <v>266</v>
       </c>
       <c r="C249">
         <v>903</v>
@@ -18692,7 +18841,7 @@
         <v>248</v>
       </c>
       <c r="B250" t="s">
-        <v>247</v>
+        <v>267</v>
       </c>
       <c r="C250">
         <v>1223</v>
@@ -18760,7 +18909,7 @@
         <v>249</v>
       </c>
       <c r="B251" t="s">
-        <v>248</v>
+        <v>268</v>
       </c>
       <c r="C251">
         <v>694</v>
@@ -18828,7 +18977,7 @@
         <v>250</v>
       </c>
       <c r="B252" t="s">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="C252">
         <v>912</v>
@@ -18896,7 +19045,7 @@
         <v>251</v>
       </c>
       <c r="B253" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C253">
         <v>1227</v>
@@ -18964,7 +19113,7 @@
         <v>252</v>
       </c>
       <c r="B254" t="s">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="C254">
         <v>961</v>
@@ -19032,7 +19181,7 @@
         <v>253</v>
       </c>
       <c r="B255" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="C255">
         <v>690</v>
@@ -19100,7 +19249,7 @@
         <v>254</v>
       </c>
       <c r="B256" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="C256">
         <v>1087</v>
@@ -19168,7 +19317,7 @@
         <v>255</v>
       </c>
       <c r="B257" t="s">
-        <v>254</v>
+        <v>274</v>
       </c>
       <c r="C257">
         <v>798</v>
@@ -19236,7 +19385,7 @@
         <v>256</v>
       </c>
       <c r="B258" t="s">
-        <v>255</v>
+        <v>275</v>
       </c>
       <c r="C258">
         <v>629</v>
@@ -19304,7 +19453,7 @@
         <v>257</v>
       </c>
       <c r="B259" t="s">
-        <v>256</v>
+        <v>276</v>
       </c>
       <c r="C259">
         <v>653</v>
@@ -19372,7 +19521,7 @@
         <v>258</v>
       </c>
       <c r="B260" t="s">
-        <v>257</v>
+        <v>277</v>
       </c>
       <c r="C260">
         <v>780</v>
@@ -19440,7 +19589,7 @@
         <v>259</v>
       </c>
       <c r="B261" t="s">
-        <v>258</v>
+        <v>278</v>
       </c>
       <c r="C261">
         <v>598</v>
@@ -19508,7 +19657,7 @@
         <v>260</v>
       </c>
       <c r="B262" t="s">
-        <v>259</v>
+        <v>279</v>
       </c>
       <c r="C262">
         <v>1161</v>
@@ -19576,7 +19725,7 @@
         <v>261</v>
       </c>
       <c r="B263" t="s">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="C263">
         <v>807</v>
@@ -19644,7 +19793,7 @@
         <v>262</v>
       </c>
       <c r="B264" t="s">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="C264">
         <v>532</v>
@@ -19712,7 +19861,7 @@
         <v>263</v>
       </c>
       <c r="B265" t="s">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="C265">
         <v>839</v>
@@ -19780,7 +19929,7 @@
         <v>264</v>
       </c>
       <c r="B266" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="C266">
         <v>783</v>
@@ -19848,7 +19997,7 @@
         <v>265</v>
       </c>
       <c r="B267" t="s">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="C267">
         <v>928</v>
@@ -19916,7 +20065,7 @@
         <v>266</v>
       </c>
       <c r="B268" t="s">
-        <v>265</v>
+        <v>285</v>
       </c>
       <c r="C268">
         <v>969</v>
@@ -19984,7 +20133,7 @@
         <v>267</v>
       </c>
       <c r="B269" t="s">
-        <v>266</v>
+        <v>286</v>
       </c>
       <c r="C269">
         <v>1113</v>
@@ -20052,7 +20201,7 @@
         <v>268</v>
       </c>
       <c r="B270" t="s">
-        <v>267</v>
+        <v>287</v>
       </c>
       <c r="C270">
         <v>1180</v>
@@ -20120,7 +20269,7 @@
         <v>269</v>
       </c>
       <c r="B271" t="s">
-        <v>268</v>
+        <v>288</v>
       </c>
       <c r="C271">
         <v>730</v>
@@ -20188,7 +20337,7 @@
         <v>270</v>
       </c>
       <c r="B272" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
       <c r="C272">
         <v>749</v>
@@ -20256,7 +20405,7 @@
         <v>271</v>
       </c>
       <c r="B273" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="C273">
         <v>1131</v>
@@ -20324,7 +20473,7 @@
         <v>272</v>
       </c>
       <c r="B274" t="s">
-        <v>271</v>
+        <v>291</v>
       </c>
       <c r="C274">
         <v>842</v>
@@ -20392,7 +20541,7 @@
         <v>273</v>
       </c>
       <c r="B275" t="s">
-        <v>272</v>
+        <v>292</v>
       </c>
       <c r="C275">
         <v>790</v>
@@ -20460,7 +20609,7 @@
         <v>274</v>
       </c>
       <c r="B276" t="s">
-        <v>273</v>
+        <v>293</v>
       </c>
       <c r="C276">
         <v>625</v>
@@ -20528,7 +20677,7 @@
         <v>275</v>
       </c>
       <c r="B277" t="s">
-        <v>274</v>
+        <v>294</v>
       </c>
       <c r="C277">
         <v>575</v>
@@ -20596,7 +20745,7 @@
         <v>276</v>
       </c>
       <c r="B278" t="s">
-        <v>275</v>
+        <v>295</v>
       </c>
       <c r="C278">
         <v>683</v>
@@ -20664,7 +20813,7 @@
         <v>277</v>
       </c>
       <c r="B279" t="s">
-        <v>276</v>
+        <v>296</v>
       </c>
       <c r="C279">
         <v>644</v>
@@ -20732,7 +20881,7 @@
         <v>278</v>
       </c>
       <c r="B280" t="s">
-        <v>277</v>
+        <v>297</v>
       </c>
       <c r="C280">
         <v>616</v>
@@ -20800,7 +20949,7 @@
         <v>279</v>
       </c>
       <c r="B281" t="s">
-        <v>278</v>
+        <v>298</v>
       </c>
       <c r="C281">
         <v>881</v>
@@ -20868,7 +21017,7 @@
         <v>280</v>
       </c>
       <c r="B282" t="s">
-        <v>279</v>
+        <v>299</v>
       </c>
       <c r="C282">
         <v>1080</v>
@@ -20936,7 +21085,7 @@
         <v>281</v>
       </c>
       <c r="B283" t="s">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="C283">
         <v>707</v>
@@ -21004,7 +21153,7 @@
         <v>282</v>
       </c>
       <c r="B284" t="s">
-        <v>281</v>
+        <v>301</v>
       </c>
       <c r="C284">
         <v>676</v>
@@ -21072,7 +21221,7 @@
         <v>283</v>
       </c>
       <c r="B285" t="s">
-        <v>282</v>
+        <v>302</v>
       </c>
       <c r="C285">
         <v>624</v>
@@ -21140,7 +21289,7 @@
         <v>284</v>
       </c>
       <c r="B286" t="s">
-        <v>283</v>
+        <v>303</v>
       </c>
       <c r="C286">
         <v>920</v>
@@ -21208,7 +21357,7 @@
         <v>285</v>
       </c>
       <c r="B287" t="s">
-        <v>284</v>
+        <v>304</v>
       </c>
       <c r="C287">
         <v>1119</v>
@@ -21276,7 +21425,7 @@
         <v>286</v>
       </c>
       <c r="B288" t="s">
-        <v>285</v>
+        <v>305</v>
       </c>
       <c r="C288">
         <v>967</v>
@@ -21344,7 +21493,7 @@
         <v>287</v>
       </c>
       <c r="B289" t="s">
-        <v>286</v>
+        <v>306</v>
       </c>
       <c r="C289">
         <v>1054</v>
@@ -21412,7 +21561,7 @@
         <v>288</v>
       </c>
       <c r="B290" t="s">
-        <v>287</v>
+        <v>307</v>
       </c>
       <c r="C290">
         <v>1168</v>
@@ -21480,7 +21629,7 @@
         <v>289</v>
       </c>
       <c r="B291" t="s">
-        <v>288</v>
+        <v>308</v>
       </c>
       <c r="C291">
         <v>1024</v>
@@ -21548,7 +21697,7 @@
         <v>290</v>
       </c>
       <c r="B292" t="s">
-        <v>289</v>
+        <v>309</v>
       </c>
       <c r="C292">
         <v>927</v>
@@ -21616,7 +21765,7 @@
         <v>291</v>
       </c>
       <c r="B293" t="s">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="C293">
         <v>873</v>
@@ -21684,7 +21833,7 @@
         <v>292</v>
       </c>
       <c r="B294" t="s">
-        <v>291</v>
+        <v>311</v>
       </c>
       <c r="C294">
         <v>933</v>
@@ -21752,7 +21901,7 @@
         <v>293</v>
       </c>
       <c r="B295" t="s">
-        <v>292</v>
+        <v>312</v>
       </c>
       <c r="C295">
         <v>874</v>
@@ -21820,7 +21969,7 @@
         <v>294</v>
       </c>
       <c r="B296" t="s">
-        <v>293</v>
+        <v>313</v>
       </c>
       <c r="C296">
         <v>820</v>
@@ -21888,7 +22037,7 @@
         <v>295</v>
       </c>
       <c r="B297" t="s">
-        <v>294</v>
+        <v>314</v>
       </c>
       <c r="C297">
         <v>821</v>
@@ -21956,7 +22105,7 @@
         <v>296</v>
       </c>
       <c r="B298" t="s">
-        <v>295</v>
+        <v>315</v>
       </c>
       <c r="C298">
         <v>1131</v>
@@ -22024,7 +22173,7 @@
         <v>297</v>
       </c>
       <c r="B299" t="s">
-        <v>296</v>
+        <v>316</v>
       </c>
       <c r="C299">
         <v>1014</v>
@@ -22092,7 +22241,7 @@
         <v>298</v>
       </c>
       <c r="B300" t="s">
-        <v>297</v>
+        <v>317</v>
       </c>
       <c r="C300">
         <v>975</v>
@@ -22160,7 +22309,7 @@
         <v>299</v>
       </c>
       <c r="B301" t="s">
-        <v>298</v>
+        <v>318</v>
       </c>
       <c r="C301">
         <v>931</v>
@@ -22228,7 +22377,7 @@
         <v>300</v>
       </c>
       <c r="B302" t="s">
-        <v>299</v>
+        <v>319</v>
       </c>
       <c r="C302">
         <v>628</v>
@@ -22296,7 +22445,7 @@
         <v>301</v>
       </c>
       <c r="B303" t="s">
-        <v>300</v>
+        <v>320</v>
       </c>
       <c r="C303">
         <v>728</v>
@@ -22364,7 +22513,7 @@
         <v>302</v>
       </c>
       <c r="B304" t="s">
-        <v>301</v>
+        <v>321</v>
       </c>
       <c r="C304">
         <v>664</v>
@@ -22432,7 +22581,7 @@
         <v>303</v>
       </c>
       <c r="B305" t="s">
-        <v>302</v>
+        <v>322</v>
       </c>
       <c r="C305">
         <v>937</v>
@@ -22500,7 +22649,7 @@
         <v>304</v>
       </c>
       <c r="B306" t="s">
-        <v>303</v>
+        <v>323</v>
       </c>
       <c r="C306">
         <v>1057</v>
@@ -22568,7 +22717,7 @@
         <v>305</v>
       </c>
       <c r="B307" t="s">
-        <v>304</v>
+        <v>324</v>
       </c>
       <c r="C307">
         <v>959</v>
@@ -22636,7 +22785,7 @@
         <v>306</v>
       </c>
       <c r="B308" t="s">
-        <v>305</v>
+        <v>325</v>
       </c>
       <c r="C308">
         <v>844</v>
@@ -22704,7 +22853,7 @@
         <v>307</v>
       </c>
       <c r="B309" t="s">
-        <v>306</v>
+        <v>326</v>
       </c>
       <c r="C309">
         <v>1140</v>
@@ -22772,7 +22921,7 @@
         <v>308</v>
       </c>
       <c r="B310" t="s">
-        <v>307</v>
+        <v>327</v>
       </c>
       <c r="C310">
         <v>855</v>
@@ -22840,7 +22989,7 @@
         <v>309</v>
       </c>
       <c r="B311" t="s">
-        <v>308</v>
+        <v>328</v>
       </c>
       <c r="C311">
         <v>316</v>
@@ -22908,7 +23057,7 @@
         <v>310</v>
       </c>
       <c r="B312" t="s">
-        <v>309</v>
+        <v>329</v>
       </c>
       <c r="C312">
         <v>690</v>
@@ -22976,7 +23125,7 @@
         <v>311</v>
       </c>
       <c r="B313" t="s">
-        <v>310</v>
+        <v>330</v>
       </c>
       <c r="C313">
         <v>728</v>
@@ -23044,7 +23193,7 @@
         <v>312</v>
       </c>
       <c r="B314" t="s">
-        <v>311</v>
+        <v>331</v>
       </c>
       <c r="C314">
         <v>796</v>
@@ -23112,7 +23261,7 @@
         <v>313</v>
       </c>
       <c r="B315" t="s">
-        <v>312</v>
+        <v>332</v>
       </c>
       <c r="C315">
         <v>626</v>
@@ -23180,7 +23329,7 @@
         <v>314</v>
       </c>
       <c r="B316" t="s">
-        <v>313</v>
+        <v>333</v>
       </c>
       <c r="C316">
         <v>661</v>
@@ -23248,7 +23397,7 @@
         <v>315</v>
       </c>
       <c r="B317" t="s">
-        <v>314</v>
+        <v>334</v>
       </c>
       <c r="C317">
         <v>828</v>
@@ -23316,7 +23465,7 @@
         <v>316</v>
       </c>
       <c r="B318" t="s">
-        <v>315</v>
+        <v>335</v>
       </c>
       <c r="C318">
         <v>876</v>
@@ -23384,7 +23533,7 @@
         <v>317</v>
       </c>
       <c r="B319" t="s">
-        <v>316</v>
+        <v>336</v>
       </c>
       <c r="C319">
         <v>1099</v>
@@ -23452,7 +23601,7 @@
         <v>318</v>
       </c>
       <c r="B320" t="s">
-        <v>317</v>
+        <v>337</v>
       </c>
       <c r="C320">
         <v>774</v>
@@ -23520,7 +23669,7 @@
         <v>319</v>
       </c>
       <c r="B321" t="s">
-        <v>318</v>
+        <v>338</v>
       </c>
       <c r="C321">
         <v>803</v>
@@ -23588,7 +23737,7 @@
         <v>320</v>
       </c>
       <c r="B322" t="s">
-        <v>319</v>
+        <v>339</v>
       </c>
       <c r="C322">
         <v>620</v>
@@ -23656,7 +23805,7 @@
         <v>321</v>
       </c>
       <c r="B323" t="s">
-        <v>320</v>
+        <v>340</v>
       </c>
       <c r="C323">
         <v>614</v>
@@ -23724,7 +23873,7 @@
         <v>322</v>
       </c>
       <c r="B324" t="s">
-        <v>321</v>
+        <v>341</v>
       </c>
       <c r="C324">
         <v>1092</v>
@@ -23792,7 +23941,7 @@
         <v>323</v>
       </c>
       <c r="B325" t="s">
-        <v>322</v>
+        <v>342</v>
       </c>
       <c r="C325">
         <v>1045</v>
@@ -23860,7 +24009,7 @@
         <v>324</v>
       </c>
       <c r="B326" t="s">
-        <v>323</v>
+        <v>343</v>
       </c>
       <c r="C326">
         <v>1184</v>
@@ -23928,7 +24077,7 @@
         <v>325</v>
       </c>
       <c r="B327" t="s">
-        <v>324</v>
+        <v>344</v>
       </c>
       <c r="C327">
         <v>1055</v>
@@ -23996,7 +24145,7 @@
         <v>326</v>
       </c>
       <c r="B328" t="s">
-        <v>325</v>
+        <v>345</v>
       </c>
       <c r="C328">
         <v>864</v>
@@ -24064,7 +24213,7 @@
         <v>327</v>
       </c>
       <c r="B329" t="s">
-        <v>326</v>
+        <v>346</v>
       </c>
       <c r="C329">
         <v>1111</v>
@@ -24132,7 +24281,7 @@
         <v>328</v>
       </c>
       <c r="B330" t="s">
-        <v>327</v>
+        <v>347</v>
       </c>
       <c r="C330">
         <v>942</v>
@@ -24200,7 +24349,7 @@
         <v>329</v>
       </c>
       <c r="B331" t="s">
-        <v>328</v>
+        <v>348</v>
       </c>
       <c r="C331">
         <v>635</v>
@@ -24268,7 +24417,7 @@
         <v>330</v>
       </c>
       <c r="B332" t="s">
-        <v>329</v>
+        <v>349</v>
       </c>
       <c r="C332">
         <v>755</v>
@@ -24336,7 +24485,7 @@
         <v>331</v>
       </c>
       <c r="B333" t="s">
-        <v>330</v>
+        <v>350</v>
       </c>
       <c r="C333">
         <v>767</v>
@@ -24404,7 +24553,7 @@
         <v>332</v>
       </c>
       <c r="B334" t="s">
-        <v>331</v>
+        <v>351</v>
       </c>
       <c r="C334">
         <v>1180</v>
@@ -24472,7 +24621,7 @@
         <v>333</v>
       </c>
       <c r="B335" t="s">
-        <v>332</v>
+        <v>352</v>
       </c>
       <c r="C335">
         <v>678</v>
@@ -24540,7 +24689,7 @@
         <v>334</v>
       </c>
       <c r="B336" t="s">
-        <v>333</v>
+        <v>353</v>
       </c>
       <c r="C336">
         <v>637</v>
@@ -24608,7 +24757,7 @@
         <v>335</v>
       </c>
       <c r="B337" t="s">
-        <v>334</v>
+        <v>354</v>
       </c>
       <c r="C337">
         <v>982</v>
@@ -24676,7 +24825,7 @@
         <v>336</v>
       </c>
       <c r="B338" t="s">
-        <v>335</v>
+        <v>355</v>
       </c>
       <c r="C338">
         <v>752</v>
@@ -24744,7 +24893,7 @@
         <v>337</v>
       </c>
       <c r="B339" t="s">
-        <v>336</v>
+        <v>356</v>
       </c>
       <c r="C339">
         <v>1217</v>
@@ -24812,7 +24961,7 @@
         <v>338</v>
       </c>
       <c r="B340" t="s">
-        <v>337</v>
+        <v>357</v>
       </c>
       <c r="C340">
         <v>585</v>
@@ -24880,7 +25029,7 @@
         <v>339</v>
       </c>
       <c r="B341" t="s">
-        <v>338</v>
+        <v>358</v>
       </c>
       <c r="C341">
         <v>1144</v>
@@ -24948,7 +25097,7 @@
         <v>340</v>
       </c>
       <c r="B342" t="s">
-        <v>339</v>
+        <v>359</v>
       </c>
       <c r="C342">
         <v>556</v>
@@ -25016,7 +25165,7 @@
         <v>341</v>
       </c>
       <c r="B343" t="s">
-        <v>340</v>
+        <v>360</v>
       </c>
       <c r="C343">
         <v>917</v>
@@ -25084,7 +25233,7 @@
         <v>342</v>
       </c>
       <c r="B344" t="s">
-        <v>341</v>
+        <v>361</v>
       </c>
       <c r="C344">
         <v>853</v>
@@ -25152,7 +25301,7 @@
         <v>343</v>
       </c>
       <c r="B345" t="s">
-        <v>342</v>
+        <v>362</v>
       </c>
       <c r="C345">
         <v>886</v>
@@ -25220,7 +25369,7 @@
         <v>344</v>
       </c>
       <c r="B346" t="s">
-        <v>343</v>
+        <v>363</v>
       </c>
       <c r="C346">
         <v>773</v>
@@ -25288,7 +25437,7 @@
         <v>345</v>
       </c>
       <c r="B347" t="s">
-        <v>344</v>
+        <v>364</v>
       </c>
       <c r="C347">
         <v>816</v>
@@ -25356,7 +25505,7 @@
         <v>346</v>
       </c>
       <c r="B348" t="s">
-        <v>345</v>
+        <v>365</v>
       </c>
       <c r="C348">
         <v>897</v>
@@ -25424,7 +25573,7 @@
         <v>347</v>
       </c>
       <c r="B349" t="s">
-        <v>346</v>
+        <v>366</v>
       </c>
       <c r="C349">
         <v>633</v>
@@ -25492,7 +25641,7 @@
         <v>348</v>
       </c>
       <c r="B350" t="s">
-        <v>347</v>
+        <v>367</v>
       </c>
       <c r="C350">
         <v>751</v>
@@ -25560,7 +25709,7 @@
         <v>349</v>
       </c>
       <c r="B351" t="s">
-        <v>348</v>
+        <v>368</v>
       </c>
       <c r="C351">
         <v>928</v>
@@ -25628,7 +25777,7 @@
         <v>350</v>
       </c>
       <c r="B352" t="s">
-        <v>349</v>
+        <v>369</v>
       </c>
       <c r="C352">
         <v>453</v>
@@ -25696,7 +25845,7 @@
         <v>351</v>
       </c>
       <c r="B353" t="s">
-        <v>350</v>
+        <v>370</v>
       </c>
       <c r="C353">
         <v>857</v>
@@ -25764,7 +25913,7 @@
         <v>352</v>
       </c>
       <c r="B354" t="s">
-        <v>351</v>
+        <v>371</v>
       </c>
       <c r="C354">
         <v>881</v>
@@ -25832,7 +25981,7 @@
         <v>353</v>
       </c>
       <c r="B355" t="s">
-        <v>352</v>
+        <v>372</v>
       </c>
       <c r="C355">
         <v>1022</v>
@@ -25900,7 +26049,7 @@
         <v>354</v>
       </c>
       <c r="B356" t="s">
-        <v>353</v>
+        <v>373</v>
       </c>
       <c r="C356">
         <v>1065</v>
@@ -25968,7 +26117,7 @@
         <v>355</v>
       </c>
       <c r="B357" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
       <c r="C357">
         <v>1139</v>
@@ -26036,7 +26185,7 @@
         <v>356</v>
       </c>
       <c r="B358" t="s">
-        <v>355</v>
+        <v>375</v>
       </c>
       <c r="C358">
         <v>723</v>
@@ -26104,7 +26253,7 @@
         <v>357</v>
       </c>
       <c r="B359" t="s">
-        <v>356</v>
+        <v>376</v>
       </c>
       <c r="C359">
         <v>1052</v>
@@ -26172,7 +26321,7 @@
         <v>358</v>
       </c>
       <c r="B360" t="s">
-        <v>357</v>
+        <v>377</v>
       </c>
       <c r="C360">
         <v>1154</v>
@@ -26240,7 +26389,7 @@
         <v>359</v>
       </c>
       <c r="B361" t="s">
-        <v>358</v>
+        <v>378</v>
       </c>
       <c r="C361">
         <v>1073</v>
@@ -26308,7 +26457,7 @@
         <v>360</v>
       </c>
       <c r="B362" t="s">
-        <v>359</v>
+        <v>379</v>
       </c>
       <c r="C362">
         <v>1083</v>
@@ -26376,7 +26525,7 @@
         <v>361</v>
       </c>
       <c r="B363" t="s">
-        <v>360</v>
+        <v>380</v>
       </c>
       <c r="C363">
         <v>670</v>
@@ -26444,7 +26593,7 @@
         <v>362</v>
       </c>
       <c r="B364" t="s">
-        <v>361</v>
+        <v>381</v>
       </c>
       <c r="C364">
         <v>651</v>
@@ -26512,7 +26661,7 @@
         <v>363</v>
       </c>
       <c r="B365" t="s">
-        <v>362</v>
+        <v>382</v>
       </c>
       <c r="C365">
         <v>1134</v>
@@ -26580,7 +26729,7 @@
         <v>364</v>
       </c>
       <c r="B366" t="s">
-        <v>363</v>
+        <v>383</v>
       </c>
       <c r="C366">
         <v>985</v>
@@ -26648,7 +26797,7 @@
         <v>365</v>
       </c>
       <c r="B367" t="s">
-        <v>364</v>
+        <v>384</v>
       </c>
       <c r="C367">
         <v>1156</v>
@@ -26716,7 +26865,7 @@
         <v>366</v>
       </c>
       <c r="B368" t="s">
-        <v>274</v>
+        <v>294</v>
       </c>
       <c r="C368">
         <v>629</v>
@@ -26784,7 +26933,7 @@
         <v>367</v>
       </c>
       <c r="B369" t="s">
-        <v>365</v>
+        <v>385</v>
       </c>
       <c r="C369">
         <v>622</v>
@@ -26852,7 +27001,7 @@
         <v>368</v>
       </c>
       <c r="B370" t="s">
-        <v>366</v>
+        <v>386</v>
       </c>
       <c r="C370">
         <v>1136</v>
@@ -26920,7 +27069,7 @@
         <v>369</v>
       </c>
       <c r="B371" t="s">
-        <v>367</v>
+        <v>387</v>
       </c>
       <c r="C371">
         <v>1058</v>
@@ -26988,7 +27137,7 @@
         <v>370</v>
       </c>
       <c r="B372" t="s">
-        <v>368</v>
+        <v>388</v>
       </c>
       <c r="C372">
         <v>924</v>
@@ -27056,7 +27205,7 @@
         <v>371</v>
       </c>
       <c r="B373" t="s">
-        <v>369</v>
+        <v>389</v>
       </c>
       <c r="C373">
         <v>873</v>
@@ -27124,7 +27273,7 @@
         <v>372</v>
       </c>
       <c r="B374" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="C374">
         <v>983</v>
@@ -27192,7 +27341,7 @@
         <v>373</v>
       </c>
       <c r="B375" t="s">
-        <v>370</v>
+        <v>390</v>
       </c>
       <c r="C375">
         <v>1016</v>
@@ -27260,7 +27409,7 @@
         <v>374</v>
       </c>
       <c r="B376" t="s">
-        <v>371</v>
+        <v>391</v>
       </c>
       <c r="C376">
         <v>1065</v>
@@ -27328,7 +27477,7 @@
         <v>375</v>
       </c>
       <c r="B377" t="s">
-        <v>372</v>
+        <v>392</v>
       </c>
       <c r="C377">
         <v>1013</v>
@@ -27396,7 +27545,7 @@
         <v>376</v>
       </c>
       <c r="B378" t="s">
-        <v>373</v>
+        <v>393</v>
       </c>
       <c r="C378">
         <v>597</v>
@@ -27464,7 +27613,7 @@
         <v>377</v>
       </c>
       <c r="B379" t="s">
-        <v>374</v>
+        <v>394</v>
       </c>
       <c r="C379">
         <v>773</v>
@@ -27532,7 +27681,7 @@
         <v>378</v>
       </c>
       <c r="B380" t="s">
-        <v>375</v>
+        <v>395</v>
       </c>
       <c r="C380">
         <v>1186</v>
@@ -27600,7 +27749,7 @@
         <v>379</v>
       </c>
       <c r="B381" t="s">
-        <v>376</v>
+        <v>396</v>
       </c>
       <c r="C381">
         <v>801</v>
@@ -27668,7 +27817,7 @@
         <v>380</v>
       </c>
       <c r="B382" t="s">
-        <v>377</v>
+        <v>397</v>
       </c>
       <c r="C382">
         <v>880</v>
@@ -27736,7 +27885,7 @@
         <v>381</v>
       </c>
       <c r="B383" t="s">
-        <v>378</v>
+        <v>398</v>
       </c>
       <c r="C383">
         <v>1048</v>
@@ -27804,7 +27953,7 @@
         <v>382</v>
       </c>
       <c r="B384" t="s">
-        <v>379</v>
+        <v>399</v>
       </c>
       <c r="C384">
         <v>995</v>
@@ -27872,7 +28021,7 @@
         <v>383</v>
       </c>
       <c r="B385" t="s">
-        <v>380</v>
+        <v>400</v>
       </c>
       <c r="C385">
         <v>703</v>
@@ -27940,7 +28089,7 @@
         <v>384</v>
       </c>
       <c r="B386" t="s">
-        <v>381</v>
+        <v>401</v>
       </c>
       <c r="C386">
         <v>1001</v>
@@ -28008,7 +28157,7 @@
         <v>385</v>
       </c>
       <c r="B387" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="C387">
         <v>1108</v>
@@ -28076,7 +28225,7 @@
         <v>386</v>
       </c>
       <c r="B388" t="s">
-        <v>383</v>
+        <v>403</v>
       </c>
       <c r="C388">
         <v>514</v>
@@ -28144,7 +28293,7 @@
         <v>387</v>
       </c>
       <c r="B389" t="s">
-        <v>384</v>
+        <v>404</v>
       </c>
       <c r="C389">
         <v>1151</v>
@@ -28212,7 +28361,7 @@
         <v>388</v>
       </c>
       <c r="B390" t="s">
-        <v>385</v>
+        <v>405</v>
       </c>
       <c r="C390">
         <v>853</v>
@@ -28280,7 +28429,7 @@
         <v>389</v>
       </c>
       <c r="B391" t="s">
-        <v>386</v>
+        <v>406</v>
       </c>
       <c r="C391">
         <v>1088</v>
@@ -28348,7 +28497,7 @@
         <v>390</v>
       </c>
       <c r="B392" t="s">
-        <v>387</v>
+        <v>407</v>
       </c>
       <c r="C392">
         <v>1005</v>
@@ -28416,7 +28565,7 @@
         <v>391</v>
       </c>
       <c r="B393" t="s">
-        <v>388</v>
+        <v>408</v>
       </c>
       <c r="C393">
         <v>1045</v>
@@ -28484,7 +28633,7 @@
         <v>392</v>
       </c>
       <c r="B394" t="s">
-        <v>389</v>
+        <v>409</v>
       </c>
       <c r="C394">
         <v>1094</v>
@@ -28552,7 +28701,7 @@
         <v>393</v>
       </c>
       <c r="B395" t="s">
-        <v>390</v>
+        <v>410</v>
       </c>
       <c r="C395">
         <v>476</v>
@@ -28620,7 +28769,7 @@
         <v>394</v>
       </c>
       <c r="B396" t="s">
-        <v>391</v>
+        <v>411</v>
       </c>
       <c r="C396">
         <v>779</v>
@@ -28688,7 +28837,7 @@
         <v>395</v>
       </c>
       <c r="B397" t="s">
-        <v>392</v>
+        <v>412</v>
       </c>
       <c r="C397">
         <v>685</v>
@@ -28756,7 +28905,7 @@
         <v>396</v>
       </c>
       <c r="B398" t="s">
-        <v>393</v>
+        <v>413</v>
       </c>
       <c r="C398">
         <v>653</v>
@@ -28824,7 +28973,7 @@
         <v>397</v>
       </c>
       <c r="B399" t="s">
-        <v>394</v>
+        <v>414</v>
       </c>
       <c r="C399">
         <v>1037</v>
@@ -28892,7 +29041,7 @@
         <v>398</v>
       </c>
       <c r="B400" t="s">
-        <v>395</v>
+        <v>415</v>
       </c>
       <c r="C400">
         <v>1132</v>
@@ -28960,7 +29109,7 @@
         <v>399</v>
       </c>
       <c r="B401" t="s">
-        <v>396</v>
+        <v>416</v>
       </c>
       <c r="C401">
         <v>1132</v>
@@ -29028,7 +29177,7 @@
         <v>400</v>
       </c>
       <c r="B402" t="s">
-        <v>397</v>
+        <v>417</v>
       </c>
       <c r="C402">
         <v>594</v>
@@ -29096,7 +29245,7 @@
         <v>401</v>
       </c>
       <c r="B403" t="s">
-        <v>398</v>
+        <v>418</v>
       </c>
       <c r="C403">
         <v>910</v>
@@ -29164,7 +29313,7 @@
         <v>402</v>
       </c>
       <c r="B404" t="s">
-        <v>399</v>
+        <v>419</v>
       </c>
       <c r="C404">
         <v>975</v>
@@ -29232,7 +29381,7 @@
         <v>403</v>
       </c>
       <c r="B405" t="s">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="C405">
         <v>658</v>
@@ -29300,7 +29449,7 @@
         <v>404</v>
       </c>
       <c r="B406" t="s">
-        <v>401</v>
+        <v>421</v>
       </c>
       <c r="C406">
         <v>760</v>
@@ -29368,7 +29517,7 @@
         <v>405</v>
       </c>
       <c r="B407" t="s">
-        <v>402</v>
+        <v>422</v>
       </c>
       <c r="C407">
         <v>1109</v>
@@ -29436,7 +29585,7 @@
         <v>406</v>
       </c>
       <c r="B408" t="s">
-        <v>403</v>
+        <v>423</v>
       </c>
       <c r="C408">
         <v>902</v>
@@ -29504,7 +29653,7 @@
         <v>407</v>
       </c>
       <c r="B409" t="s">
-        <v>404</v>
+        <v>424</v>
       </c>
       <c r="C409">
         <v>1040</v>
@@ -29572,7 +29721,7 @@
         <v>408</v>
       </c>
       <c r="B410" t="s">
-        <v>405</v>
+        <v>425</v>
       </c>
       <c r="C410">
         <v>866</v>
@@ -29640,7 +29789,7 @@
         <v>409</v>
       </c>
       <c r="B411" t="s">
-        <v>406</v>
+        <v>426</v>
       </c>
       <c r="C411">
         <v>850</v>
@@ -29708,7 +29857,7 @@
         <v>410</v>
       </c>
       <c r="B412" t="s">
-        <v>407</v>
+        <v>427</v>
       </c>
       <c r="C412">
         <v>706</v>
@@ -29776,7 +29925,7 @@
         <v>411</v>
       </c>
       <c r="B413" t="s">
-        <v>408</v>
+        <v>428</v>
       </c>
       <c r="C413">
         <v>900</v>
@@ -29844,7 +29993,7 @@
         <v>412</v>
       </c>
       <c r="B414" t="s">
-        <v>409</v>
+        <v>429</v>
       </c>
       <c r="C414">
         <v>1044</v>
@@ -29912,7 +30061,7 @@
         <v>413</v>
       </c>
       <c r="B415" t="s">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="C415">
         <v>1002</v>
@@ -29980,7 +30129,7 @@
         <v>414</v>
       </c>
       <c r="B416" t="s">
-        <v>411</v>
+        <v>431</v>
       </c>
       <c r="C416">
         <v>1069</v>
@@ -30048,7 +30197,7 @@
         <v>415</v>
       </c>
       <c r="B417" t="s">
-        <v>412</v>
+        <v>432</v>
       </c>
       <c r="C417">
         <v>849</v>
@@ -30116,7 +30265,7 @@
         <v>416</v>
       </c>
       <c r="B418" t="s">
-        <v>413</v>
+        <v>433</v>
       </c>
       <c r="C418">
         <v>943</v>
@@ -30184,7 +30333,7 @@
         <v>417</v>
       </c>
       <c r="B419" t="s">
-        <v>414</v>
+        <v>434</v>
       </c>
       <c r="C419">
         <v>1244</v>
@@ -30252,7 +30401,7 @@
         <v>418</v>
       </c>
       <c r="B420" t="s">
-        <v>415</v>
+        <v>435</v>
       </c>
       <c r="C420">
         <v>1226</v>
@@ -30320,7 +30469,7 @@
         <v>419</v>
       </c>
       <c r="B421" t="s">
-        <v>416</v>
+        <v>436</v>
       </c>
       <c r="C421">
         <v>1087</v>
@@ -30388,7 +30537,7 @@
         <v>420</v>
       </c>
       <c r="B422" t="s">
-        <v>417</v>
+        <v>437</v>
       </c>
       <c r="C422">
         <v>1203</v>
@@ -30456,7 +30605,7 @@
         <v>421</v>
       </c>
       <c r="B423" t="s">
-        <v>417</v>
+        <v>437</v>
       </c>
       <c r="C423">
         <v>1060</v>
@@ -30524,7 +30673,7 @@
         <v>422</v>
       </c>
       <c r="B424" t="s">
-        <v>418</v>
+        <v>438</v>
       </c>
       <c r="C424">
         <v>1044</v>
@@ -30592,7 +30741,7 @@
         <v>423</v>
       </c>
       <c r="B425" t="s">
-        <v>419</v>
+        <v>439</v>
       </c>
       <c r="C425">
         <v>802</v>
@@ -30660,7 +30809,7 @@
         <v>424</v>
       </c>
       <c r="B426" t="s">
-        <v>420</v>
+        <v>440</v>
       </c>
       <c r="C426">
         <v>855</v>
@@ -30728,7 +30877,7 @@
         <v>425</v>
       </c>
       <c r="B427" t="s">
-        <v>421</v>
+        <v>441</v>
       </c>
       <c r="C427">
         <v>1093</v>
@@ -30796,7 +30945,7 @@
         <v>426</v>
       </c>
       <c r="B428" t="s">
-        <v>422</v>
+        <v>442</v>
       </c>
       <c r="C428">
         <v>1062</v>
@@ -30864,7 +31013,7 @@
         <v>427</v>
       </c>
       <c r="B429" t="s">
-        <v>423</v>
+        <v>443</v>
       </c>
       <c r="C429">
         <v>879</v>
@@ -30932,7 +31081,7 @@
         <v>428</v>
       </c>
       <c r="B430" t="s">
-        <v>424</v>
+        <v>444</v>
       </c>
       <c r="C430">
         <v>922</v>
@@ -31000,7 +31149,7 @@
         <v>429</v>
       </c>
       <c r="B431" t="s">
-        <v>425</v>
+        <v>445</v>
       </c>
       <c r="C431">
         <v>929</v>
@@ -31068,7 +31217,7 @@
         <v>430</v>
       </c>
       <c r="B432" t="s">
-        <v>426</v>
+        <v>446</v>
       </c>
       <c r="C432">
         <v>1197</v>
@@ -31136,7 +31285,7 @@
         <v>431</v>
       </c>
       <c r="B433" t="s">
-        <v>427</v>
+        <v>447</v>
       </c>
       <c r="C433">
         <v>804</v>
@@ -31204,7 +31353,7 @@
         <v>432</v>
       </c>
       <c r="B434" t="s">
-        <v>428</v>
+        <v>448</v>
       </c>
       <c r="C434">
         <v>762</v>
@@ -31272,7 +31421,7 @@
         <v>433</v>
       </c>
       <c r="B435" t="s">
-        <v>429</v>
+        <v>449</v>
       </c>
       <c r="C435">
         <v>715</v>
@@ -31340,7 +31489,7 @@
         <v>434</v>
       </c>
       <c r="B436" t="s">
-        <v>430</v>
+        <v>450</v>
       </c>
       <c r="C436">
         <v>767</v>
@@ -31408,7 +31557,7 @@
         <v>435</v>
       </c>
       <c r="B437" t="s">
-        <v>431</v>
+        <v>451</v>
       </c>
       <c r="C437">
         <v>1197</v>
@@ -31476,7 +31625,7 @@
         <v>436</v>
       </c>
       <c r="B438" t="s">
-        <v>432</v>
+        <v>452</v>
       </c>
       <c r="C438">
         <v>657</v>
@@ -31544,7 +31693,7 @@
         <v>437</v>
       </c>
       <c r="B439" t="s">
-        <v>433</v>
+        <v>453</v>
       </c>
       <c r="C439">
         <v>783</v>
@@ -31612,7 +31761,7 @@
         <v>438</v>
       </c>
       <c r="B440" t="s">
-        <v>434</v>
+        <v>454</v>
       </c>
       <c r="C440">
         <v>722</v>
@@ -31680,7 +31829,7 @@
         <v>439</v>
       </c>
       <c r="B441" t="s">
-        <v>435</v>
+        <v>455</v>
       </c>
       <c r="C441">
         <v>696</v>
@@ -31748,7 +31897,7 @@
         <v>440</v>
       </c>
       <c r="B442" t="s">
-        <v>436</v>
+        <v>456</v>
       </c>
       <c r="C442">
         <v>949</v>
@@ -31816,7 +31965,7 @@
         <v>441</v>
       </c>
       <c r="B443" t="s">
-        <v>437</v>
+        <v>457</v>
       </c>
       <c r="C443">
         <v>880</v>
@@ -31884,7 +32033,7 @@
         <v>442</v>
       </c>
       <c r="B444" t="s">
-        <v>438</v>
+        <v>458</v>
       </c>
       <c r="C444">
         <v>896</v>
@@ -31952,7 +32101,7 @@
         <v>443</v>
       </c>
       <c r="B445" t="s">
-        <v>439</v>
+        <v>459</v>
       </c>
       <c r="C445">
         <v>1184</v>
@@ -32020,7 +32169,7 @@
         <v>444</v>
       </c>
       <c r="B446" t="s">
-        <v>440</v>
+        <v>460</v>
       </c>
       <c r="C446">
         <v>900</v>
@@ -32088,7 +32237,7 @@
         <v>445</v>
       </c>
       <c r="B447" t="s">
-        <v>441</v>
+        <v>461</v>
       </c>
       <c r="C447">
         <v>857</v>
@@ -32156,7 +32305,7 @@
         <v>446</v>
       </c>
       <c r="B448" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="C448">
         <v>1118</v>
@@ -32224,7 +32373,7 @@
         <v>447</v>
       </c>
       <c r="B449" t="s">
-        <v>443</v>
+        <v>463</v>
       </c>
       <c r="C449">
         <v>710</v>
@@ -32292,7 +32441,7 @@
         <v>448</v>
       </c>
       <c r="B450" t="s">
-        <v>444</v>
+        <v>464</v>
       </c>
       <c r="C450">
         <v>670</v>
@@ -32360,7 +32509,7 @@
         <v>449</v>
       </c>
       <c r="B451" t="s">
-        <v>445</v>
+        <v>465</v>
       </c>
       <c r="C451">
         <v>808</v>
@@ -32428,7 +32577,7 @@
         <v>450</v>
       </c>
       <c r="B452" t="s">
-        <v>446</v>
+        <v>466</v>
       </c>
       <c r="C452">
         <v>462</v>
@@ -32496,7 +32645,7 @@
         <v>451</v>
       </c>
       <c r="B453" t="s">
-        <v>447</v>
+        <v>467</v>
       </c>
       <c r="C453">
         <v>1196</v>
@@ -32564,7 +32713,7 @@
         <v>452</v>
       </c>
       <c r="B454" t="s">
-        <v>448</v>
+        <v>468</v>
       </c>
       <c r="C454">
         <v>361</v>
@@ -32632,7 +32781,7 @@
         <v>453</v>
       </c>
       <c r="B455" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="C455">
         <v>1160</v>
@@ -32700,7 +32849,7 @@
         <v>454</v>
       </c>
       <c r="B456" t="s">
-        <v>450</v>
+        <v>470</v>
       </c>
       <c r="C456">
         <v>1111</v>
@@ -32768,7 +32917,7 @@
         <v>455</v>
       </c>
       <c r="B457" t="s">
-        <v>451</v>
+        <v>471</v>
       </c>
       <c r="C457">
         <v>889</v>
@@ -32836,7 +32985,7 @@
         <v>456</v>
       </c>
       <c r="B458" t="s">
-        <v>452</v>
+        <v>472</v>
       </c>
       <c r="C458">
         <v>827</v>
@@ -32904,7 +33053,7 @@
         <v>457</v>
       </c>
       <c r="B459" t="s">
-        <v>453</v>
+        <v>473</v>
       </c>
       <c r="C459">
         <v>926</v>
@@ -32972,7 +33121,7 @@
         <v>458</v>
       </c>
       <c r="B460" t="s">
-        <v>454</v>
+        <v>474</v>
       </c>
       <c r="C460">
         <v>1057</v>
@@ -33040,7 +33189,7 @@
         <v>459</v>
       </c>
       <c r="B461" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="C461">
         <v>1083</v>
@@ -33108,7 +33257,7 @@
         <v>460</v>
       </c>
       <c r="B462" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
       <c r="C462">
         <v>488</v>
@@ -33176,7 +33325,7 @@
         <v>461</v>
       </c>
       <c r="B463" t="s">
-        <v>457</v>
+        <v>477</v>
       </c>
       <c r="C463">
         <v>1092</v>
@@ -33244,7 +33393,7 @@
         <v>462</v>
       </c>
       <c r="B464" t="s">
-        <v>458</v>
+        <v>478</v>
       </c>
       <c r="C464">
         <v>662</v>
@@ -33312,7 +33461,7 @@
         <v>463</v>
       </c>
       <c r="B465" t="s">
-        <v>459</v>
+        <v>479</v>
       </c>
       <c r="C465">
         <v>938</v>
@@ -33380,7 +33529,7 @@
         <v>464</v>
       </c>
       <c r="B466" t="s">
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="C466">
         <v>998</v>
@@ -33448,7 +33597,7 @@
         <v>465</v>
       </c>
       <c r="B467" t="s">
-        <v>461</v>
+        <v>481</v>
       </c>
       <c r="C467">
         <v>771</v>
@@ -33516,7 +33665,7 @@
         <v>466</v>
       </c>
       <c r="B468" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="C468">
         <v>668</v>
@@ -33584,7 +33733,7 @@
         <v>467</v>
       </c>
       <c r="B469" t="s">
-        <v>463</v>
+        <v>483</v>
       </c>
       <c r="C469">
         <v>878</v>
@@ -33652,7 +33801,7 @@
         <v>468</v>
       </c>
       <c r="B470" t="s">
-        <v>464</v>
+        <v>484</v>
       </c>
       <c r="C470">
         <v>815</v>
@@ -33720,7 +33869,7 @@
         <v>469</v>
       </c>
       <c r="B471" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="C471">
         <v>820</v>
@@ -33788,7 +33937,7 @@
         <v>470</v>
       </c>
       <c r="B472" t="s">
-        <v>466</v>
+        <v>486</v>
       </c>
       <c r="C472">
         <v>308</v>
@@ -33856,7 +34005,7 @@
         <v>471</v>
       </c>
       <c r="B473" t="s">
-        <v>335</v>
+        <v>355</v>
       </c>
       <c r="C473">
         <v>784</v>
@@ -33924,7 +34073,7 @@
         <v>472</v>
       </c>
       <c r="B474" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="C474">
         <v>1072</v>
@@ -33992,7 +34141,7 @@
         <v>473</v>
       </c>
       <c r="B475" t="s">
-        <v>468</v>
+        <v>488</v>
       </c>
       <c r="C475">
         <v>1133</v>
@@ -34060,7 +34209,7 @@
         <v>474</v>
       </c>
       <c r="B476" t="s">
-        <v>469</v>
+        <v>489</v>
       </c>
       <c r="C476">
         <v>885</v>

</xml_diff>